<commit_message>
Auto commit - 03021205
</commit_message>
<xml_diff>
--- a/IM/202602_Service_Count_Report.xlsx
+++ b/IM/202602_Service_Count_Report.xlsx
@@ -3417,28 +3417,28 @@
     <t>15:12:00</t>
   </si>
   <si>
+    <t>11:19:00</t>
+  </si>
+  <si>
+    <t>THILF03853</t>
+  </si>
+  <si>
+    <t>新北市板橋區互助街48號一樓全部及50號一樓及地下室全部</t>
+  </si>
+  <si>
+    <t>板橋互助店</t>
+  </si>
+  <si>
+    <t>線路重新整理 驅動程式校正後測試正常</t>
+  </si>
+  <si>
+    <t>掃槍校正後測試正常</t>
+  </si>
+  <si>
     <t>11:17:00</t>
   </si>
   <si>
-    <t>THILF03853</t>
-  </si>
-  <si>
-    <t>新北市板橋區互助街48號一樓全部及50號一樓及地下室全部</t>
-  </si>
-  <si>
-    <t>板橋互助店</t>
-  </si>
-  <si>
     <t>PMQ1 7210002852</t>
-  </si>
-  <si>
-    <t>11:19:00</t>
-  </si>
-  <si>
-    <t>線路重新整理 驅動程式校正後測試正常</t>
-  </si>
-  <si>
-    <t>掃槍校正後測試正常</t>
   </si>
   <si>
     <t>09:38:00</t>
@@ -5525,7 +5525,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="7">
-        <v>2026021919</v>
+        <v>2026021920</v>
       </c>
       <c r="C23" s="7">
         <v>1</v>
@@ -5564,7 +5564,7 @@
         <v>94</v>
       </c>
       <c r="O23" s="7" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P23" s="7"/>
       <c r="Q23" s="7">
@@ -5573,9 +5573,7 @@
       <c r="R23" s="7">
         <v>2601</v>
       </c>
-      <c r="S23" s="7" t="s">
-        <v>41</v>
-      </c>
+      <c r="S23" s="7"/>
       <c r="T23" s="7"/>
       <c r="U23" s="7"/>
       <c r="V23" s="7"/>
@@ -5597,7 +5595,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="3">
-        <v>2026021920</v>
+        <v>2026021919</v>
       </c>
       <c r="C24" s="3">
         <v>1</v>
@@ -5636,7 +5634,7 @@
         <v>94</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P24" s="3"/>
       <c r="Q24" s="3">
@@ -5645,7 +5643,9 @@
       <c r="R24" s="3">
         <v>2601</v>
       </c>
-      <c r="S24" s="3"/>
+      <c r="S24" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="T24" s="3"/>
       <c r="U24" s="3"/>
       <c r="V24" s="3"/>
@@ -5665,7 +5665,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="7">
-        <v>2026020065</v>
+        <v>2026020064</v>
       </c>
       <c r="C25" s="7">
         <v>1</v>
@@ -5704,7 +5704,7 @@
         <v>120</v>
       </c>
       <c r="O25" s="7" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P25" s="7"/>
       <c r="Q25" s="7">
@@ -5713,7 +5713,9 @@
       <c r="R25" s="7">
         <v>16243</v>
       </c>
-      <c r="S25" s="7"/>
+      <c r="S25" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="T25" s="7"/>
       <c r="U25" s="7"/>
       <c r="V25" s="7"/>
@@ -5735,7 +5737,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="3">
-        <v>2026020064</v>
+        <v>2026020065</v>
       </c>
       <c r="C26" s="3">
         <v>1</v>
@@ -5774,7 +5776,7 @@
         <v>120</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P26" s="3"/>
       <c r="Q26" s="3">
@@ -5783,9 +5785,7 @@
       <c r="R26" s="3">
         <v>16243</v>
       </c>
-      <c r="S26" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="S26" s="3"/>
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
       <c r="V26" s="3"/>
@@ -6763,7 +6763,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="7">
-        <v>2026020521</v>
+        <v>2026020520</v>
       </c>
       <c r="C41" s="7">
         <v>1</v>
@@ -6802,14 +6802,16 @@
         <v>175</v>
       </c>
       <c r="O41" s="7" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P41" s="7"/>
       <c r="Q41" s="7"/>
       <c r="R41" s="7">
         <v>76429</v>
       </c>
-      <c r="S41" s="7"/>
+      <c r="S41" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="T41" s="7"/>
       <c r="U41" s="7"/>
       <c r="V41" s="7"/>
@@ -6831,7 +6833,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="3">
-        <v>2026020520</v>
+        <v>2026020521</v>
       </c>
       <c r="C42" s="3">
         <v>1</v>
@@ -6870,16 +6872,14 @@
         <v>175</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P42" s="3"/>
       <c r="Q42" s="3"/>
       <c r="R42" s="3">
         <v>76429</v>
       </c>
-      <c r="S42" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="S42" s="3"/>
       <c r="T42" s="3"/>
       <c r="U42" s="3"/>
       <c r="V42" s="3"/>
@@ -7637,7 +7637,7 @@
         <v>52</v>
       </c>
       <c r="B54" s="3">
-        <v>2026020807</v>
+        <v>2026020745</v>
       </c>
       <c r="C54" s="3">
         <v>1</v>
@@ -7674,16 +7674,14 @@
       </c>
       <c r="N54" s="6"/>
       <c r="O54" s="3" t="s">
-        <v>50</v>
+        <v>123</v>
       </c>
       <c r="P54" s="3"/>
       <c r="Q54" s="3"/>
       <c r="R54" s="3">
         <v>114848</v>
       </c>
-      <c r="S54" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="S54" s="3"/>
       <c r="T54" s="3"/>
       <c r="U54" s="3"/>
       <c r="V54" s="3"/>
@@ -7691,17 +7689,21 @@
       <c r="X54" s="3"/>
       <c r="Y54" s="3"/>
       <c r="Z54" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="AA54" s="3"/>
-      <c r="AB54" s="3"/>
+        <v>214</v>
+      </c>
+      <c r="AA54" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB54" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="55" spans="1:28">
       <c r="A55" s="7">
         <v>53</v>
       </c>
       <c r="B55" s="7">
-        <v>2026020808</v>
+        <v>2026020807</v>
       </c>
       <c r="C55" s="7">
         <v>1</v>
@@ -7738,14 +7740,16 @@
       </c>
       <c r="N55" s="8"/>
       <c r="O55" s="7" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P55" s="7"/>
       <c r="Q55" s="7"/>
       <c r="R55" s="7">
         <v>114848</v>
       </c>
-      <c r="S55" s="7"/>
+      <c r="S55" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="T55" s="7"/>
       <c r="U55" s="7"/>
       <c r="V55" s="7"/>
@@ -7763,7 +7767,7 @@
         <v>54</v>
       </c>
       <c r="B56" s="3">
-        <v>2026020745</v>
+        <v>2026020808</v>
       </c>
       <c r="C56" s="3">
         <v>1</v>
@@ -7800,7 +7804,7 @@
       </c>
       <c r="N56" s="6"/>
       <c r="O56" s="3" t="s">
-        <v>123</v>
+        <v>39</v>
       </c>
       <c r="P56" s="3"/>
       <c r="Q56" s="3"/>
@@ -7815,11 +7819,9 @@
       <c r="X56" s="3"/>
       <c r="Y56" s="3"/>
       <c r="Z56" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="AA56" s="3" t="s">
-        <v>41</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="AA56" s="3"/>
       <c r="AB56" s="3"/>
     </row>
     <row r="57" spans="1:28">
@@ -7961,7 +7963,7 @@
         <v>57</v>
       </c>
       <c r="B59" s="7">
-        <v>2026020810</v>
+        <v>2026020811</v>
       </c>
       <c r="C59" s="7">
         <v>1</v>
@@ -7998,16 +8000,14 @@
       </c>
       <c r="N59" s="8"/>
       <c r="O59" s="7" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P59" s="7"/>
       <c r="Q59" s="7"/>
       <c r="R59" s="7">
         <v>208475</v>
       </c>
-      <c r="S59" s="7" t="s">
-        <v>41</v>
-      </c>
+      <c r="S59" s="7"/>
       <c r="T59" s="7"/>
       <c r="U59" s="7"/>
       <c r="V59" s="7"/>
@@ -8029,7 +8029,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="3">
-        <v>2026020811</v>
+        <v>2026020810</v>
       </c>
       <c r="C60" s="3">
         <v>1</v>
@@ -8066,14 +8066,16 @@
       </c>
       <c r="N60" s="6"/>
       <c r="O60" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P60" s="3"/>
       <c r="Q60" s="3"/>
       <c r="R60" s="3">
         <v>208475</v>
       </c>
-      <c r="S60" s="3"/>
+      <c r="S60" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="T60" s="3"/>
       <c r="U60" s="3"/>
       <c r="V60" s="3"/>
@@ -8161,7 +8163,7 @@
         <v>60</v>
       </c>
       <c r="B62" s="3">
-        <v>2026021756</v>
+        <v>2026021755</v>
       </c>
       <c r="C62" s="3">
         <v>1</v>
@@ -8198,14 +8200,16 @@
       </c>
       <c r="N62" s="6"/>
       <c r="O62" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P62" s="3"/>
       <c r="Q62" s="3"/>
       <c r="R62" s="3">
         <v>229325</v>
       </c>
-      <c r="S62" s="3"/>
+      <c r="S62" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="T62" s="3"/>
       <c r="U62" s="3"/>
       <c r="V62" s="3"/>
@@ -8227,7 +8231,7 @@
         <v>61</v>
       </c>
       <c r="B63" s="7">
-        <v>2026021755</v>
+        <v>2026021756</v>
       </c>
       <c r="C63" s="7">
         <v>1</v>
@@ -8264,16 +8268,14 @@
       </c>
       <c r="N63" s="8"/>
       <c r="O63" s="7" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P63" s="7"/>
       <c r="Q63" s="7"/>
       <c r="R63" s="7">
         <v>229325</v>
       </c>
-      <c r="S63" s="7" t="s">
-        <v>41</v>
-      </c>
+      <c r="S63" s="7"/>
       <c r="T63" s="7"/>
       <c r="U63" s="7"/>
       <c r="V63" s="7"/>
@@ -13613,7 +13615,7 @@
         <v>141</v>
       </c>
       <c r="B143" s="7">
-        <v>2026022150</v>
+        <v>2026022149</v>
       </c>
       <c r="C143" s="7">
         <v>1</v>
@@ -13652,7 +13654,7 @@
         <v>537</v>
       </c>
       <c r="O143" s="7" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P143" s="7"/>
       <c r="Q143" s="7">
@@ -13661,7 +13663,9 @@
       <c r="R143" s="7">
         <v>10160</v>
       </c>
-      <c r="S143" s="7"/>
+      <c r="S143" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="T143" s="7"/>
       <c r="U143" s="7"/>
       <c r="V143" s="7"/>
@@ -13683,7 +13687,7 @@
         <v>142</v>
       </c>
       <c r="B144" s="3">
-        <v>2026022149</v>
+        <v>2026022150</v>
       </c>
       <c r="C144" s="3">
         <v>1</v>
@@ -13722,7 +13726,7 @@
         <v>537</v>
       </c>
       <c r="O144" s="3" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P144" s="3"/>
       <c r="Q144" s="3">
@@ -13731,9 +13735,7 @@
       <c r="R144" s="3">
         <v>10160</v>
       </c>
-      <c r="S144" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="S144" s="3"/>
       <c r="T144" s="3"/>
       <c r="U144" s="3"/>
       <c r="V144" s="3"/>
@@ -14025,7 +14027,7 @@
         <v>147</v>
       </c>
       <c r="B149" s="7">
-        <v>2026022158</v>
+        <v>2026022157</v>
       </c>
       <c r="C149" s="7">
         <v>1</v>
@@ -14062,14 +14064,16 @@
       </c>
       <c r="N149" s="8"/>
       <c r="O149" s="7" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P149" s="7"/>
       <c r="Q149" s="7"/>
       <c r="R149" s="7">
         <v>32194</v>
       </c>
-      <c r="S149" s="7"/>
+      <c r="S149" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="T149" s="7"/>
       <c r="U149" s="7"/>
       <c r="V149" s="7"/>
@@ -14079,19 +14083,15 @@
       <c r="Z149" s="8" t="s">
         <v>547</v>
       </c>
-      <c r="AA149" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AB149" s="7">
-        <v>1</v>
-      </c>
+      <c r="AA149" s="7"/>
+      <c r="AB149" s="7"/>
     </row>
     <row r="150" spans="1:28">
       <c r="A150" s="3">
         <v>148</v>
       </c>
       <c r="B150" s="3">
-        <v>2026022157</v>
+        <v>2026022158</v>
       </c>
       <c r="C150" s="3">
         <v>1</v>
@@ -14128,16 +14128,14 @@
       </c>
       <c r="N150" s="6"/>
       <c r="O150" s="3" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P150" s="3"/>
       <c r="Q150" s="3"/>
       <c r="R150" s="3">
         <v>32194</v>
       </c>
-      <c r="S150" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="S150" s="3"/>
       <c r="T150" s="3"/>
       <c r="U150" s="3"/>
       <c r="V150" s="3"/>
@@ -14147,7 +14145,9 @@
       <c r="Z150" s="6" t="s">
         <v>547</v>
       </c>
-      <c r="AA150" s="3"/>
+      <c r="AA150" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="AB150" s="3"/>
     </row>
     <row r="151" spans="1:28">
@@ -15907,7 +15907,7 @@
         <v>175</v>
       </c>
       <c r="B177" s="7">
-        <v>2026021649</v>
+        <v>2026021648</v>
       </c>
       <c r="C177" s="7">
         <v>1</v>
@@ -15946,7 +15946,7 @@
         <v>599</v>
       </c>
       <c r="O177" s="7" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P177" s="7"/>
       <c r="Q177" s="7">
@@ -15955,7 +15955,9 @@
       <c r="R177" s="7">
         <v>307964</v>
       </c>
-      <c r="S177" s="7"/>
+      <c r="S177" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="T177" s="7"/>
       <c r="U177" s="7"/>
       <c r="V177" s="7"/>
@@ -15973,7 +15975,7 @@
         <v>176</v>
       </c>
       <c r="B178" s="3">
-        <v>2026021648</v>
+        <v>2026021649</v>
       </c>
       <c r="C178" s="3">
         <v>1</v>
@@ -16012,7 +16014,7 @@
         <v>599</v>
       </c>
       <c r="O178" s="3" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P178" s="3"/>
       <c r="Q178" s="3">
@@ -16021,9 +16023,7 @@
       <c r="R178" s="3">
         <v>307964</v>
       </c>
-      <c r="S178" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="S178" s="3"/>
       <c r="T178" s="3"/>
       <c r="U178" s="3"/>
       <c r="V178" s="3"/>
@@ -19171,7 +19171,7 @@
         <v>224</v>
       </c>
       <c r="B226" s="3">
-        <v>2026021832</v>
+        <v>2026021831</v>
       </c>
       <c r="C226" s="3">
         <v>1</v>
@@ -19208,7 +19208,7 @@
       </c>
       <c r="N226" s="6"/>
       <c r="O226" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P226" s="3"/>
       <c r="Q226" s="3">
@@ -19217,7 +19217,9 @@
       <c r="R226" s="3">
         <v>47000</v>
       </c>
-      <c r="S226" s="3"/>
+      <c r="S226" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="T226" s="3"/>
       <c r="U226" s="3"/>
       <c r="V226" s="3"/>
@@ -19239,7 +19241,7 @@
         <v>225</v>
       </c>
       <c r="B227" s="7">
-        <v>2026021831</v>
+        <v>2026021832</v>
       </c>
       <c r="C227" s="7">
         <v>1</v>
@@ -19276,7 +19278,7 @@
       </c>
       <c r="N227" s="8"/>
       <c r="O227" s="7" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P227" s="7"/>
       <c r="Q227" s="7">
@@ -19285,9 +19287,7 @@
       <c r="R227" s="7">
         <v>47000</v>
       </c>
-      <c r="S227" s="7" t="s">
-        <v>41</v>
-      </c>
+      <c r="S227" s="7"/>
       <c r="T227" s="7"/>
       <c r="U227" s="7"/>
       <c r="V227" s="7"/>
@@ -22621,7 +22621,7 @@
         <v>274</v>
       </c>
       <c r="B276" s="3">
-        <v>2026021240</v>
+        <v>2026021239</v>
       </c>
       <c r="C276" s="3">
         <v>1</v>
@@ -22660,14 +22660,16 @@
         <v>851</v>
       </c>
       <c r="O276" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P276" s="3"/>
       <c r="Q276" s="3"/>
       <c r="R276" s="3">
         <v>51524</v>
       </c>
-      <c r="S276" s="3"/>
+      <c r="S276" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="T276" s="3"/>
       <c r="U276" s="3"/>
       <c r="V276" s="3"/>
@@ -22689,7 +22691,7 @@
         <v>275</v>
       </c>
       <c r="B277" s="7">
-        <v>2026021239</v>
+        <v>2026021240</v>
       </c>
       <c r="C277" s="7">
         <v>1</v>
@@ -22728,16 +22730,14 @@
         <v>851</v>
       </c>
       <c r="O277" s="7" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P277" s="7"/>
       <c r="Q277" s="7"/>
       <c r="R277" s="7">
         <v>51524</v>
       </c>
-      <c r="S277" s="7" t="s">
-        <v>41</v>
-      </c>
+      <c r="S277" s="7"/>
       <c r="T277" s="7"/>
       <c r="U277" s="7"/>
       <c r="V277" s="7"/>
@@ -24179,7 +24179,7 @@
         <v>297</v>
       </c>
       <c r="B299" s="7">
-        <v>2026020849</v>
+        <v>2026020850</v>
       </c>
       <c r="C299" s="7">
         <v>1</v>
@@ -24218,16 +24218,14 @@
         <v>886</v>
       </c>
       <c r="O299" s="7" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P299" s="7"/>
       <c r="Q299" s="7"/>
       <c r="R299" s="7">
         <v>16789</v>
       </c>
-      <c r="S299" s="7" t="s">
-        <v>41</v>
-      </c>
+      <c r="S299" s="7"/>
       <c r="T299" s="7"/>
       <c r="U299" s="7"/>
       <c r="V299" s="7"/>
@@ -24249,7 +24247,7 @@
         <v>298</v>
       </c>
       <c r="B300" s="3">
-        <v>2026020850</v>
+        <v>2026020849</v>
       </c>
       <c r="C300" s="3">
         <v>1</v>
@@ -24288,14 +24286,16 @@
         <v>886</v>
       </c>
       <c r="O300" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P300" s="3"/>
       <c r="Q300" s="3"/>
       <c r="R300" s="3">
         <v>16789</v>
       </c>
-      <c r="S300" s="3"/>
+      <c r="S300" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="T300" s="3"/>
       <c r="U300" s="3"/>
       <c r="V300" s="3"/>
@@ -25063,7 +25063,7 @@
         <v>310</v>
       </c>
       <c r="B312" s="3">
-        <v>2026022865</v>
+        <v>2026022864</v>
       </c>
       <c r="C312" s="3">
         <v>1</v>
@@ -25102,7 +25102,7 @@
         <v>904</v>
       </c>
       <c r="O312" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P312" s="3"/>
       <c r="Q312" s="3">
@@ -25111,7 +25111,9 @@
       <c r="R312" s="3">
         <v>5861</v>
       </c>
-      <c r="S312" s="3"/>
+      <c r="S312" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="T312" s="3"/>
       <c r="U312" s="3"/>
       <c r="V312" s="3"/>
@@ -25121,19 +25123,15 @@
       <c r="Z312" s="6" t="s">
         <v>783</v>
       </c>
-      <c r="AA312" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="AB312" s="3">
-        <v>1</v>
-      </c>
+      <c r="AA312" s="3"/>
+      <c r="AB312" s="3"/>
     </row>
     <row r="313" spans="1:28">
       <c r="A313" s="7">
         <v>311</v>
       </c>
       <c r="B313" s="7">
-        <v>2026022864</v>
+        <v>2026022865</v>
       </c>
       <c r="C313" s="7">
         <v>1</v>
@@ -25172,7 +25170,7 @@
         <v>904</v>
       </c>
       <c r="O313" s="7" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P313" s="7"/>
       <c r="Q313" s="7">
@@ -25181,9 +25179,7 @@
       <c r="R313" s="7">
         <v>5861</v>
       </c>
-      <c r="S313" s="7" t="s">
-        <v>41</v>
-      </c>
+      <c r="S313" s="7"/>
       <c r="T313" s="7"/>
       <c r="U313" s="7"/>
       <c r="V313" s="7"/>
@@ -25193,7 +25189,9 @@
       <c r="Z313" s="8" t="s">
         <v>783</v>
       </c>
-      <c r="AA313" s="7"/>
+      <c r="AA313" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="AB313" s="7"/>
     </row>
     <row r="314" spans="1:28">
@@ -25811,7 +25809,7 @@
         <v>321</v>
       </c>
       <c r="B323" s="7">
-        <v>2026021465</v>
+        <v>2026021464</v>
       </c>
       <c r="C323" s="7">
         <v>1</v>
@@ -25850,14 +25848,16 @@
         <v>917</v>
       </c>
       <c r="O323" s="7" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P323" s="7"/>
       <c r="Q323" s="7"/>
       <c r="R323" s="7">
         <v>7717</v>
       </c>
-      <c r="S323" s="7"/>
+      <c r="S323" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="T323" s="7"/>
       <c r="U323" s="7"/>
       <c r="V323" s="7"/>
@@ -25867,19 +25867,15 @@
       <c r="Z323" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="AA323" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AB323" s="7">
-        <v>1</v>
-      </c>
+      <c r="AA323" s="7"/>
+      <c r="AB323" s="7"/>
     </row>
     <row r="324" spans="1:28">
       <c r="A324" s="3">
         <v>322</v>
       </c>
       <c r="B324" s="3">
-        <v>2026021464</v>
+        <v>2026021465</v>
       </c>
       <c r="C324" s="3">
         <v>1</v>
@@ -25918,16 +25914,14 @@
         <v>917</v>
       </c>
       <c r="O324" s="3" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P324" s="3"/>
       <c r="Q324" s="3"/>
       <c r="R324" s="3">
         <v>7717</v>
       </c>
-      <c r="S324" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="S324" s="3"/>
       <c r="T324" s="3"/>
       <c r="U324" s="3"/>
       <c r="V324" s="3"/>
@@ -25937,7 +25931,9 @@
       <c r="Z324" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="AA324" s="3"/>
+      <c r="AA324" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="AB324" s="3"/>
     </row>
     <row r="325" spans="1:28">
@@ -31491,7 +31487,7 @@
         <v>405</v>
       </c>
       <c r="B407" s="7">
-        <v>2026022852</v>
+        <v>2026022853</v>
       </c>
       <c r="C407" s="7">
         <v>1</v>
@@ -31530,16 +31526,14 @@
         <v>1101</v>
       </c>
       <c r="O407" s="7" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P407" s="7"/>
       <c r="Q407" s="7"/>
       <c r="R407" s="7">
         <v>6740</v>
       </c>
-      <c r="S407" s="7" t="s">
-        <v>41</v>
-      </c>
+      <c r="S407" s="7"/>
       <c r="T407" s="7"/>
       <c r="U407" s="7"/>
       <c r="V407" s="7"/>
@@ -31549,15 +31543,19 @@
       <c r="Z407" s="8" t="s">
         <v>783</v>
       </c>
-      <c r="AA407" s="7"/>
-      <c r="AB407" s="7"/>
+      <c r="AA407" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB407" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="408" spans="1:28">
       <c r="A408" s="3">
         <v>406</v>
       </c>
       <c r="B408" s="3">
-        <v>2026022853</v>
+        <v>2026022852</v>
       </c>
       <c r="C408" s="3">
         <v>1</v>
@@ -31596,14 +31594,16 @@
         <v>1101</v>
       </c>
       <c r="O408" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P408" s="3"/>
       <c r="Q408" s="3"/>
       <c r="R408" s="3">
         <v>6740</v>
       </c>
-      <c r="S408" s="3"/>
+      <c r="S408" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="T408" s="3"/>
       <c r="U408" s="3"/>
       <c r="V408" s="3"/>
@@ -31613,9 +31613,7 @@
       <c r="Z408" s="6" t="s">
         <v>783</v>
       </c>
-      <c r="AA408" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="AA408" s="3"/>
       <c r="AB408" s="3"/>
     </row>
     <row r="409" spans="1:28">
@@ -31623,7 +31621,7 @@
         <v>407</v>
       </c>
       <c r="B409" s="7">
-        <v>2026022851</v>
+        <v>2026022850</v>
       </c>
       <c r="C409" s="7">
         <v>1</v>
@@ -31662,14 +31660,16 @@
         <v>1104</v>
       </c>
       <c r="O409" s="7" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="P409" s="7"/>
       <c r="Q409" s="7"/>
       <c r="R409" s="7">
         <v>3983</v>
       </c>
-      <c r="S409" s="7"/>
+      <c r="S409" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="T409" s="7"/>
       <c r="U409" s="7"/>
       <c r="V409" s="7"/>
@@ -31679,19 +31679,15 @@
       <c r="Z409" s="8" t="s">
         <v>783</v>
       </c>
-      <c r="AA409" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AB409" s="7">
-        <v>1</v>
-      </c>
+      <c r="AA409" s="7"/>
+      <c r="AB409" s="7"/>
     </row>
     <row r="410" spans="1:28">
       <c r="A410" s="3">
         <v>408</v>
       </c>
       <c r="B410" s="3">
-        <v>2026022850</v>
+        <v>2026022851</v>
       </c>
       <c r="C410" s="3">
         <v>1</v>
@@ -31730,16 +31726,14 @@
         <v>1104</v>
       </c>
       <c r="O410" s="3" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P410" s="3"/>
       <c r="Q410" s="3"/>
       <c r="R410" s="3">
         <v>3983</v>
       </c>
-      <c r="S410" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="S410" s="3"/>
       <c r="T410" s="3"/>
       <c r="U410" s="3"/>
       <c r="V410" s="3"/>
@@ -31749,7 +31743,9 @@
       <c r="Z410" s="6" t="s">
         <v>783</v>
       </c>
-      <c r="AA410" s="3"/>
+      <c r="AA410" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="AB410" s="3"/>
     </row>
     <row r="411" spans="1:28">
@@ -32029,7 +32025,7 @@
         <v>413</v>
       </c>
       <c r="B415" s="7">
-        <v>2026021655</v>
+        <v>2026021432</v>
       </c>
       <c r="C415" s="7">
         <v>1</v>
@@ -32052,8 +32048,12 @@
       <c r="I415" s="7" t="s">
         <v>1113</v>
       </c>
-      <c r="J415" s="7"/>
-      <c r="K415" s="7"/>
+      <c r="J415" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="K415" s="7" t="s">
+        <v>262</v>
+      </c>
       <c r="L415" s="8" t="s">
         <v>257</v>
       </c>
@@ -32064,16 +32064,14 @@
         <v>1115</v>
       </c>
       <c r="O415" s="7" t="s">
-        <v>50</v>
+        <v>123</v>
       </c>
       <c r="P415" s="7"/>
       <c r="Q415" s="7"/>
       <c r="R415" s="7">
         <v>0</v>
       </c>
-      <c r="S415" s="7" t="s">
-        <v>41</v>
-      </c>
+      <c r="S415" s="7"/>
       <c r="T415" s="7"/>
       <c r="U415" s="7"/>
       <c r="V415" s="7"/>
@@ -32083,15 +32081,19 @@
       <c r="Z415" s="8" t="s">
         <v>1116</v>
       </c>
-      <c r="AA415" s="7"/>
-      <c r="AB415" s="7"/>
+      <c r="AA415" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB415" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="416" spans="1:28">
       <c r="A416" s="3">
         <v>414</v>
       </c>
       <c r="B416" s="3">
-        <v>2026021432</v>
+        <v>2026021433</v>
       </c>
       <c r="C416" s="3">
         <v>1</v>
@@ -32109,7 +32111,7 @@
         <v>271</v>
       </c>
       <c r="H416" s="3" t="s">
-        <v>1117</v>
+        <v>1112</v>
       </c>
       <c r="I416" s="3" t="s">
         <v>1113</v>
@@ -32145,7 +32147,7 @@
       <c r="X416" s="3"/>
       <c r="Y416" s="3"/>
       <c r="Z416" s="6" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="AA416" s="3" t="s">
         <v>41</v>
@@ -32157,7 +32159,7 @@
         <v>415</v>
       </c>
       <c r="B417" s="7">
-        <v>2026021433</v>
+        <v>2026021434</v>
       </c>
       <c r="C417" s="7">
         <v>1</v>
@@ -32175,7 +32177,7 @@
         <v>271</v>
       </c>
       <c r="H417" s="7" t="s">
-        <v>1117</v>
+        <v>376</v>
       </c>
       <c r="I417" s="7" t="s">
         <v>1113</v>
@@ -32211,7 +32213,7 @@
       <c r="X417" s="7"/>
       <c r="Y417" s="7"/>
       <c r="Z417" s="8" t="s">
-        <v>1119</v>
+        <v>1117</v>
       </c>
       <c r="AA417" s="7" t="s">
         <v>41</v>
@@ -32223,7 +32225,7 @@
         <v>416</v>
       </c>
       <c r="B418" s="3">
-        <v>2026021434</v>
+        <v>2026021655</v>
       </c>
       <c r="C418" s="3">
         <v>1</v>
@@ -32241,17 +32243,13 @@
         <v>271</v>
       </c>
       <c r="H418" s="3" t="s">
-        <v>376</v>
+        <v>1118</v>
       </c>
       <c r="I418" s="3" t="s">
         <v>1113</v>
       </c>
-      <c r="J418" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="K418" s="3" t="s">
-        <v>262</v>
-      </c>
+      <c r="J418" s="3"/>
+      <c r="K418" s="3"/>
       <c r="L418" s="6" t="s">
         <v>257</v>
       </c>
@@ -32262,14 +32260,16 @@
         <v>1115</v>
       </c>
       <c r="O418" s="3" t="s">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="P418" s="3"/>
       <c r="Q418" s="3"/>
       <c r="R418" s="3">
         <v>0</v>
       </c>
-      <c r="S418" s="3"/>
+      <c r="S418" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="T418" s="3"/>
       <c r="U418" s="3"/>
       <c r="V418" s="3"/>
@@ -32279,9 +32279,7 @@
       <c r="Z418" s="6" t="s">
         <v>1119</v>
       </c>
-      <c r="AA418" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="AA418" s="3"/>
       <c r="AB418" s="3"/>
     </row>
     <row r="419" spans="1:28">
@@ -33107,7 +33105,7 @@
         <v>1160</v>
       </c>
       <c r="AB431" s="9">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>